<commit_message>
Update state maps 2026-03-27
</commit_message>
<xml_diff>
--- a/epr-tracker.xlsx
+++ b/epr-tracker.xlsx
@@ -538,7 +538,7 @@
       </c>
       <c r="D2" s="4" t="inlineStr"/>
       <c r="E2" s="4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
@@ -630,7 +630,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr"/>
       <c r="E6" s="4" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
@@ -656,7 +656,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr"/>
       <c r="E7" s="4" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
@@ -682,7 +682,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr"/>
       <c r="E8" s="4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
@@ -704,7 +704,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr"/>
       <c r="E9" s="4" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
@@ -748,7 +748,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr"/>
       <c r="E11" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
@@ -818,7 +818,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr"/>
       <c r="E14" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
@@ -844,7 +844,7 @@
       </c>
       <c r="D15" s="4" t="inlineStr"/>
       <c r="E15" s="4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
@@ -958,7 +958,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr"/>
       <c r="E20" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
@@ -1010,7 +1010,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr"/>
       <c r="E22" s="4" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
@@ -1032,7 +1032,7 @@
       </c>
       <c r="D23" s="4" t="inlineStr"/>
       <c r="E23" s="4" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
@@ -1058,7 +1058,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr"/>
       <c r="E24" s="4" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -1080,7 +1080,7 @@
       </c>
       <c r="D25" s="4" t="inlineStr"/>
       <c r="E25" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
@@ -1124,7 +1124,7 @@
       </c>
       <c r="D27" s="4" t="inlineStr"/>
       <c r="E27" s="4" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr"/>
       <c r="E32" s="4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
@@ -1260,7 +1260,7 @@
       </c>
       <c r="D33" s="4" t="inlineStr"/>
       <c r="E33" s="4" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
@@ -1282,7 +1282,7 @@
       </c>
       <c r="D34" s="4" t="inlineStr"/>
       <c r="E34" s="4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       </c>
       <c r="D35" s="4" t="inlineStr"/>
       <c r="E35" s="4" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
@@ -1378,7 +1378,7 @@
       </c>
       <c r="D38" s="4" t="inlineStr"/>
       <c r="E38" s="4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
@@ -1400,7 +1400,7 @@
       </c>
       <c r="D39" s="4" t="inlineStr"/>
       <c r="E39" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
@@ -1426,7 +1426,7 @@
       </c>
       <c r="D40" s="4" t="inlineStr"/>
       <c r="E40" s="4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
       </c>
       <c r="D41" s="4" t="inlineStr"/>
       <c r="E41" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
@@ -1492,7 +1492,7 @@
       </c>
       <c r="D43" s="4" t="inlineStr"/>
       <c r="E43" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
@@ -1558,7 +1558,7 @@
       </c>
       <c r="D46" s="4" t="inlineStr"/>
       <c r="E46" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
@@ -1584,7 +1584,7 @@
       </c>
       <c r="D47" s="4" t="inlineStr"/>
       <c r="E47" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
@@ -1610,7 +1610,7 @@
       </c>
       <c r="D48" s="4" t="inlineStr"/>
       <c r="E48" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
@@ -1632,7 +1632,7 @@
       </c>
       <c r="D49" s="4" t="inlineStr"/>
       <c r="E49" s="4" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
@@ -1654,7 +1654,7 @@
       </c>
       <c r="D50" s="4" t="inlineStr"/>
       <c r="E50" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
@@ -1676,7 +1676,7 @@
       </c>
       <c r="D51" s="4" t="inlineStr"/>
       <c r="E51" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>

</xml_diff>